<commit_message>
PED_hourly_dispatch_data.csv Bulk update: input data, PED disptch code and disptch outputs
</commit_message>
<xml_diff>
--- a/app/modules/common/AD/F16_input/DH_technology_cost.xlsx
+++ b/app/modules/common/AD/F16_input/DH_technology_cost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20375"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hasani\Documents\Workplace\Dispatch Guide\Neuer Ordner\Dispatch\app\modules\common\AD\F16_input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tuwienacat-my.sharepoint.com/personal/nirav_patel_tuwien_ac_at/Documents/Desktop/PED_SupplyOptimization/hotmapsDispatch/app/modules/common/AD/F16_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1070FF-B6D4-44C0-A8FE-D264DD68A5AE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{FB1070FF-B6D4-44C0-A8FE-D264DD68A5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED54221A-AEE6-49EA-B4EF-9A978B944A0F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="780" windowWidth="29040" windowHeight="15990" tabRatio="869" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25710" yWindow="4200" windowWidth="25820" windowHeight="13900" tabRatio="869" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Heat Generators" sheetId="1" r:id="rId1"/>
@@ -736,7 +736,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -798,8 +798,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
@@ -810,10 +809,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Eingabe" xfId="3" builtinId="20"/>
-    <cellStyle name="Gut" xfId="1" builtinId="26"/>
-    <cellStyle name="Schlecht" xfId="2" builtinId="27"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Input" xfId="3" builtinId="20"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -829,9 +828,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -869,9 +868,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -904,26 +903,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -956,26 +938,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1150,34 +1115,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.86328125" customWidth="1"/>
+    <col min="3" max="3" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.1328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.3984375" customWidth="1"/>
+    <col min="11" max="11" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.3984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.59765625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" s="8" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="9" t="s">
         <v>14</v>
       </c>
@@ -1263,7 +1228,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="10" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" s="10" customFormat="1" ht="114" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>14</v>
       </c>
@@ -1349,7 +1314,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1415,7 +1380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
@@ -1481,7 +1446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
@@ -1547,7 +1512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
@@ -1613,7 +1578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
         <v>1</v>
       </c>
@@ -1679,7 +1644,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
         <v>0</v>
       </c>
@@ -1745,7 +1710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
         <v>87</v>
       </c>
@@ -1811,7 +1776,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
         <v>88</v>
       </c>
@@ -1877,7 +1842,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
         <v>88</v>
       </c>
@@ -1943,7 +1908,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
         <v>88</v>
       </c>
@@ -2009,7 +1974,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
         <v>88</v>
       </c>
@@ -2075,7 +2040,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
         <v>88</v>
       </c>
@@ -2141,7 +2106,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
         <v>87</v>
       </c>
@@ -2207,7 +2172,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
         <v>87</v>
       </c>
@@ -2273,7 +2238,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
         <v>88</v>
       </c>
@@ -2339,7 +2304,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
         <v>87</v>
       </c>
@@ -2405,7 +2370,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A19" s="13" t="s">
         <v>61</v>
       </c>
@@ -2471,7 +2436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A20" s="18" t="s">
         <v>82</v>
       </c>
@@ -2555,7 +2520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A21" s="18" t="s">
         <v>82</v>
       </c>
@@ -2639,7 +2604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A22" s="18" t="s">
         <v>82</v>
       </c>
@@ -2723,7 +2688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A23" s="18" t="s">
         <v>112</v>
       </c>
@@ -2799,7 +2764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A24" s="18" t="s">
         <v>98</v>
       </c>
@@ -2883,7 +2848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A25" s="18" t="s">
         <v>98</v>
       </c>
@@ -2950,7 +2915,7 @@
       <c r="V25" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="W25" s="27"/>
+      <c r="W25" s="25"/>
       <c r="X25" s="18">
         <v>0</v>
       </c>
@@ -2967,7 +2932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A26" s="18" t="s">
         <v>98</v>
       </c>
@@ -3051,7 +3016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A27" s="18" t="s">
         <v>99</v>
       </c>
@@ -3135,7 +3100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A28" s="18" t="s">
         <v>99</v>
       </c>
@@ -3219,7 +3184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A29" s="18" t="s">
         <v>99</v>
       </c>
@@ -3303,7 +3268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A30" s="18" t="s">
         <v>97</v>
       </c>
@@ -3387,7 +3352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A31" s="18" t="s">
         <v>97</v>
       </c>
@@ -3471,7 +3436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.45">
       <c r="A32" s="18" t="s">
         <v>97</v>
       </c>
@@ -3564,15 +3529,15 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEAEE1BE-767B-4768-81E9-7BCEA9DC4038}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>153</v>
       </c>
@@ -3586,7 +3551,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -3609,7 +3574,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -3632,7 +3597,7 @@
         <v>2.77</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -3655,7 +3620,7 @@
         <v>2.71</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -3678,7 +3643,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -3701,7 +3666,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -3724,7 +3689,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -3747,7 +3712,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>
@@ -3778,15 +3743,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14F39DA3-EBB6-4252-93BB-F99777A8976E}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>154</v>
       </c>
@@ -3800,7 +3765,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -3820,7 +3785,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3840,7 +3805,7 @@
         <v>1.99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -3860,7 +3825,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -3888,14 +3853,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE56874-8322-48E0-BD03-05EBF58D3817}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.3984375" customWidth="1"/>
+    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>155</v>
       </c>
@@ -3909,7 +3874,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -3926,7 +3891,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3943,7 +3908,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -3960,7 +3925,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -3985,14 +3950,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14153C57-D390-42EF-8A65-6CD4C93BD32C}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.59765625" customWidth="1"/>
+    <col min="2" max="2" width="22.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>153</v>
       </c>
@@ -4006,7 +3971,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4029,7 +3994,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -4052,7 +4017,7 @@
         <v>2.77</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -4075,7 +4040,7 @@
         <v>2.71</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -4098,7 +4063,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -4121,7 +4086,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -4144,7 +4109,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -4167,7 +4132,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>
@@ -4198,14 +4163,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D98414A-455A-4234-B72F-5DB50D746BD9}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>154</v>
       </c>
@@ -4219,7 +4184,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4239,7 +4204,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4259,7 +4224,7 @@
         <v>1.99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4279,7 +4244,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -4307,14 +4272,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD26C3C0-AC1D-47AD-BA98-3B15BC973534}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.3984375" customWidth="1"/>
+    <col min="2" max="2" width="22.1328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>155</v>
       </c>
@@ -4328,7 +4293,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4345,7 +4310,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4362,7 +4327,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4379,7 +4344,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -4404,14 +4369,14 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E4E640D-2AAC-4A6C-BE86-CDD8335BFD60}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.59765625" customWidth="1"/>
+    <col min="2" max="2" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>153</v>
       </c>
@@ -4425,7 +4390,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4448,7 +4413,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -4471,7 +4436,7 @@
         <v>2.77</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -4494,7 +4459,7 @@
         <v>2.71</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -4517,7 +4482,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -4540,7 +4505,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -4563,7 +4528,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -4586,7 +4551,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>
@@ -4617,14 +4582,14 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00E862EE-497C-4CCA-9A03-E7317EDF542D}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>154</v>
       </c>
@@ -4638,7 +4603,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4658,7 +4623,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4678,7 +4643,7 @@
         <v>1.99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4698,7 +4663,7 @@
         <v>1.96</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -4726,14 +4691,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F350A461-0808-4E13-B075-55CFBDDAB3DA}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.3984375" customWidth="1"/>
+    <col min="2" max="2" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>155</v>
       </c>
@@ -4747,7 +4712,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -4764,7 +4729,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -4781,7 +4746,7 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4798,7 +4763,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -4823,14 +4788,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.140625" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1328125" customWidth="1"/>
+    <col min="2" max="2" width="20.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
         <v>34</v>
       </c>
@@ -4841,7 +4806,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="12" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A2" s="11" t="s">
         <v>25</v>
       </c>
@@ -4852,7 +4817,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -4860,65 +4825,65 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>0.24299999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>164</v>
       </c>
       <c r="B5" s="4">
-        <v>62</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="C5">
+        <v>0.22700000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="4">
-        <v>47</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="C6">
+        <v>0.26700000000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="5">
-        <v>30</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="C7">
+        <v>0.20200000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="4">
-        <v>22</v>
+        <v>65</v>
       </c>
       <c r="C8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -4926,10 +4891,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
@@ -4937,10 +4902,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -4948,10 +4913,10 @@
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
@@ -4959,32 +4924,32 @@
         <v>0</v>
       </c>
       <c r="C12" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B13" s="4">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="C13" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="4">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="C14" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>42</v>
       </c>
@@ -4995,10 +4960,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A16" s="27"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -5008,17 +4973,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="9" t="s">
         <v>40</v>
       </c>
@@ -5038,7 +5003,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>91</v>
       </c>
@@ -5058,7 +5023,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>25</v>
       </c>
@@ -5086,21 +5051,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+    <col min="1" max="1" width="24.3984375" customWidth="1"/>
+    <col min="2" max="2" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.59765625" customWidth="1"/>
     <col min="4" max="4" width="32" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.59765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.3984375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
         <v>50</v>
       </c>
@@ -5132,7 +5097,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="11" t="s">
         <v>16</v>
       </c>
@@ -5164,7 +5129,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>96</v>
       </c>
@@ -5205,77 +5170,77 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="18" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" s="18" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" s="18" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" s="18" t="s">
         <v>112</v>
       </c>
@@ -5289,15 +5254,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.59765625" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>148</v>
       </c>
@@ -5311,7 +5276,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="17" t="s">
         <v>69</v>
       </c>
@@ -5334,7 +5299,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -5357,7 +5322,7 @@
         <v>9.49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -5380,7 +5345,7 @@
         <v>10.210000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -5403,7 +5368,7 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -5426,7 +5391,7 @@
         <v>9.0399999999999991</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -5449,7 +5414,7 @@
         <v>7.28</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -5472,7 +5437,7 @@
         <v>4.72</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>
@@ -5504,13 +5469,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="2" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1328125" customWidth="1"/>
+    <col min="2" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>150</v>
       </c>
@@ -5524,7 +5489,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="16" t="s">
         <v>69</v>
       </c>
@@ -5547,7 +5512,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="16" t="s">
         <v>76</v>
       </c>
@@ -5570,7 +5535,7 @@
         <v>3.27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="16" t="s">
         <v>77</v>
       </c>
@@ -5593,7 +5558,7 @@
         <v>3.15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="16" t="s">
         <v>78</v>
       </c>
@@ -5616,7 +5581,7 @@
         <v>3.09</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="16" t="s">
         <v>79</v>
       </c>
@@ -5639,7 +5604,7 @@
         <v>2.98</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="16" t="s">
         <v>80</v>
       </c>
@@ -5662,7 +5627,7 @@
         <v>2.87</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="16" t="s">
         <v>81</v>
       </c>
@@ -5685,7 +5650,7 @@
         <v>2.65</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="16" t="s">
         <v>70</v>
       </c>
@@ -5716,13 +5681,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>148</v>
       </c>
@@ -5736,7 +5701,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -5759,7 +5724,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -5782,7 +5747,7 @@
         <v>2.5299999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -5805,7 +5770,7 @@
         <v>2.48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -5828,7 +5793,7 @@
         <v>2.4300000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -5851,7 +5816,7 @@
         <v>2.38</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -5874,7 +5839,7 @@
         <v>2.3199999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -5897,7 +5862,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>
@@ -5928,14 +5893,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>148</v>
       </c>
@@ -5949,7 +5914,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -5972,7 +5937,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -5995,7 +5960,7 @@
         <v>2.77</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -6018,7 +5983,7 @@
         <v>2.71</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -6041,7 +6006,7 @@
         <v>2.66</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -6064,7 +6029,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -6087,7 +6052,7 @@
         <v>2.5499999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -6110,7 +6075,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>70</v>
       </c>

</xml_diff>